<commit_message>
Added comparison to synergy package and added to test suite
</commit_message>
<xml_diff>
--- a/outputs/RKO/parameters/Dinaciclib_parameters.xlsx
+++ b/outputs/RKO/parameters/Dinaciclib_parameters.xlsx
@@ -428,7 +428,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.590865399784002e-17</v>
+        <v>4.00294172137627e-23</v>
       </c>
     </row>
     <row r="3">
@@ -438,7 +438,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9736843028178734</v>
+        <v>0.9736840183934813</v>
       </c>
     </row>
     <row r="4">
@@ -448,7 +448,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.01337353464173423</v>
+        <v>0.01337356415191069</v>
       </c>
     </row>
     <row r="5">
@@ -458,7 +458,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.197765138360452</v>
+        <v>2.197774386076497</v>
       </c>
     </row>
   </sheetData>

</xml_diff>